<commit_message>
Leads: automatische Quellen-Verifikation + 18 weitere Logistik-Leads
- verify_leads.py ruft je Lead die angegebene Quell-URL ab und sucht die
  Adresse woertlich im HTML (inkl. Cloudflare-Verschleierung und
  URL-kodierten mailto-Links); Ergebnis landet als _verifiziert im Rohdatum
- build_leads.py nimmt nur noch bestaetigte Adressen in die Tabelle auf
- Logistik & Supply Chain: 25 Leads, alle 25 gegen ihre Quelle bestaetigt

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011LNRMjEMhsYjaDQzNDCkTb
</commit_message>
<xml_diff>
--- a/leads-adept/leads-adept.xlsx
+++ b/leads-adept/leads-adept.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Verworfen" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$I$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$I$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -544,27 +544,27 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Anja Hollenhorst</t>
+          <t>Wolfgang Heidel</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Geschäftsführerin (lt. Impressum; auf der Website Ansprechpartnerin Kundenservice)</t>
+          <t>Geschäftsleitung</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>anja@hti-spedition.de</t>
+          <t>wolfgang.heidel@bayern-express-spedition.de</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>+49 251 74787-0 (Zentrale, Durchwahlen 11-21)</t>
+          <t>+49 89 329892-10</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>HTI Spedition und Logistik GmbH</t>
+          <t>Bayern Express Spedition GmbH</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -574,44 +574,44 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Münster (NRW)</t>
+          <t>Garching bei München, weiterer Standort Pilsting-Ganacker, Bayern</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Familiengeführte Spedition (Familie Hollenhorst) mit Fernverkehr, Luft-/Seefracht inkl. Zollabwicklung, Lager und Status Reglementierter Beauftragter. Zoll-, Fracht- und Dispositionsprozesse mit hohem Dokumentenaufkommen — gutes Feld für Prozessautomatisierung und Systemanbindung.</t>
+          <t>Familiengeführte bayerische Spedition (Familie Heidel) mit Fernverkehr, Nahverkehrsdisposition, Stückgut-/VTL-Systemverkehr und eigener Abwicklung an zwei Standorten.</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>https://hti-spedition.de/ | https://hti-spedition.de/impressum/</t>
+          <t>https://www.bayern-express-spedition.de/mitarbeiter.php</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Florian Meyer</t>
+          <t>Jens Haverland</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Geschäftsführung / Logistik- und Lagerleitung</t>
+          <t>Geschäftsführer</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>florian.meyer@rdllogistik.de</t>
+          <t>jhaverland@cargomar.de</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>+49 (0)2151 36806-16</t>
+          <t>+49 421 5590-10 (Zentrale)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>RDL Logistik Rheinische Distributions- und Lagerlogistik GmbH</t>
+          <t>Cargomar GmbH Internationale Spedition / Cargomar Air &amp; Sea GmbH</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -621,44 +621,44 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Krefeld (Niederrhein, NRW), zweiter Standort Willich</t>
+          <t>Bremen</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Inhabergeführter Lager- und Distributionslogistiker am Niederrhein (seit 2000) mit Lagerlogistik, Distribution und Fuhrpark an zwei Standorten. Geschäftsführung leitet operativ Lager und Abrechnung selbst — Digitalisierung von Lagerverwaltung, Disposition und Abrechnung ist unmittelbar chef-relevant.</t>
+          <t>Inhabergeführte Bremer Spedition mit See-/Luftfracht, Import/Export sowie eigener Lagerlogistik (Teamleitung Lagerlogistik im Haus).</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>https://rdllogistik.de/ueber-uns/ | https://rdllogistik.de/ | https://rdllogistik.de/impressum/</t>
+          <t>https://www.cargomar.de/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Michael Hoeper</t>
+          <t>Dr. Rimbert J. Kelber</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Geschäftsführer</t>
+          <t>Niederlassungsleitung</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>hoeper@hoeper-spedition.de</t>
+          <t>rimbert.kelber@koester-hapke-sped.com</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>02862-418327-10</t>
+          <t>+49 5132 822-100</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Richard Hoeper GmbH &amp; Co. KG (Hoeper Spedition)</t>
+          <t>Carl Köster &amp; Louis Hapke GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -668,44 +668,44 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Südlohn-Oeding (Westmünsterland, NRW)</t>
+          <t>Sehnde-Höver bei Hannover, Niedersachsen</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Familienunternehmen in zweiter Generation mit Transporten, eigenem Fuhrpark, Lagerlogistik und Palettenmanagement im Westmünsterland. Kleinerer, aber voll ausgebauter Betrieb mit Dispo-, QM- und Projektmanagement-Funktionen; Hinweis: liegt vermutlich unterhalb der 50-Mitarbeiter-Schwelle.</t>
+          <t>Mittelständische, inhabergeführte Spedition seit 1854 mit nationalen/internationalen Stückgutverkehren, Messelogistik und eigener Lagerlogistik (eigene Lagerleitung).</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>https://hoeper-spedition.de/team/ | https://hoeper-spedition.de/ | https://hoeper-spedition.de/impressum/</t>
+          <t>https://koester-hapke-sped.com/ansprechpartner/ | https://koester-hapke-sped.com/wir-ueber-uns/ | https://koester-hapke-sped.com/kontakt/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Bernd Häger</t>
+          <t>Anja Hollenhorst</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Geschäftsführer</t>
+          <t>Geschäftsführerin (lt. Impressum; auf der Website Ansprechpartnerin Kundenservice)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>bhaeger@spedition-haeger.de</t>
+          <t>anja@hti-spedition.de</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>02904 9740-0</t>
+          <t>+49 251 74787-0 (Zentrale, Durchwahlen 11-21)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Spedition Häger GmbH &amp; Co. KG / Häger Transporte u. Logistik GmbH &amp; Co. KG</t>
+          <t>HTI Spedition und Logistik GmbH</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -715,44 +715,44 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Bestwig (Sauerland, NRW)</t>
+          <t>Münster (NRW)</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Familiengeführte Sauerland-Spedition mit Transport-, Lager- und Kontraktlogistik über zwei Schwestergesellschaften. Zwei-Firmen-Struktur und gewachsene Dispositions-/Lagerprozesse sprechen für manuelle Abläufe mit Digitalisierungs- und Systemintegrationsbedarf.</t>
+          <t>Familiengeführte Spedition (Familie Hollenhorst) mit Fernverkehr, Luft-/Seefracht inkl. Zollabwicklung, Lager und Status Reglementierter Beauftragter. Zoll-, Fracht- und Dispositionsprozesse mit hohem Dokumentenaufkommen — gutes Feld für Prozessautomatisierung und Systemanbindung.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>https://www.spedition-haeger.de/kontakt/</t>
+          <t>https://hti-spedition.de/ | https://hti-spedition.de/impressum/</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Theodor Schulz</t>
+          <t>Peter Plank</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Geschäftsführer (Disposition &amp; Kundenbetreuung)</t>
+          <t>Vorsitzender Geschäftsführer / Inhaber</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>ts@schulz-spedition.de</t>
+          <t>peterplank@hellmold-plank.de</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>+49 251 26333-211</t>
+          <t>+49 641 95201-16</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Theodor Schulz GmbH &amp; Co. KG (Schulz Spedition)</t>
+          <t>Hellmold &amp; Plank GmbH &amp; Co. KG Spedition</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -762,69 +762,915 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Münster (NRW)</t>
+          <t>Gießen (Europastr. 7+9, 35394), Hessen</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Inhabergeführte Münsteraner Spedition mit Transport, Lagerung/Lagerverwaltung, Palettenmanagement und Abrechnung als eigene Abteilungen. Geschäftsführung sitzt selbst in der Disposition — kurze Entscheidungswege, viele manuell getriebene Dispo- und Abrechnungsprozesse als Digitalisierungsansatz.</t>
+          <t>1904 gegründete, inhabergeführte hessische Spedition (seit 1996 im Alleinbesitz der Familie Plank) mit Systemverkehren, Fernverkehr und Lagerlogistik; zweite Generation (Niklas Plank) in der Geschäftsführung.</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>https://www.schulz-spedition.de/ | https://www.schulz-spedition.de/#unternehmen</t>
+          <t>https://www.hellmold-plank.de/de/kontakt | https://www.hellmold-plank.de/</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>Ingo Kaiser</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Geschäftsführung (Management)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>ingo.kaiser@ikg-spedition.de</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>+49 7223 281689-19</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>IKG Spedition GmbH</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Baden-Baden / Sinzheim, Baden-Württemberg</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Familiengeführte Spedition (Ingo und Kristina Kaiser) mit intermodalen Transporten Richtung Italien/Frankreich/Schweiz, eigenem Lager und Fuhrpark sowie Niederlassung in Busto Arsizio.</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ikg-spedition.de/team/ | https://www.ikg-spedition.de/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Joachim Berends</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>j.berends@bentheimer-eisenbahn.de</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>+49 5921 8034-0</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Kraftverkehr Emsland GmbH</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Nordhorn, Niedersachsen</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Geschäftsführer der Kraftverkehr Emsland GmbH (Spedition/Logistiklager der Bentheimer Eisenbahn-Gruppe). Hinweis: die auf der Ansprechpartner-Seite genannte E-Mail läuft über die Domain der Muttergesellschaft.</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kraftverkehr-emsland.de/kontakt/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Marco Oppermann</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Speditionsleitung &amp; Prokurist</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>marco.oppermann@kraftverkehr-emsland.de</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>+49 5921 8034-96</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Kraftverkehr Emsland GmbH</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Nordhorn, Niedersachsen</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Mittelständische Spedition mit Sammelgut, Ladungsverkehren und eigenem Warehousing-Bereich; Prokurist und Speditionsleiter mit Entscheidungsbefugnis über Prozesse/IT-Themen.</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kraftverkehr-emsland.de/kontakt/ | https://www.kraftverkehr-emsland.de/spedition-logistiklager/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Florian Meyer</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Geschäftsführung / Logistik- und Lagerleitung</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>florian.meyer@rdllogistik.de</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>+49 (0)2151 36806-16</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>RDL Logistik Rheinische Distributions- und Lagerlogistik GmbH</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Krefeld (Niederrhein, NRW), zweiter Standort Willich</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Inhabergeführter Lager- und Distributionslogistiker am Niederrhein (seit 2000) mit Lagerlogistik, Distribution und Fuhrpark an zwei Standorten. Geschäftsführung leitet operativ Lager und Abrechnung selbst — Digitalisierung von Lagerverwaltung, Disposition und Abrechnung ist unmittelbar chef-relevant.</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>https://rdllogistik.de/ueber-uns/ | https://rdllogistik.de/ | https://rdllogistik.de/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Michael Hoeper</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>hoeper@hoeper-spedition.de</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>02862-418327-10</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Richard Hoeper GmbH &amp; Co. KG (Hoeper Spedition)</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Südlohn-Oeding (Westmünsterland, NRW)</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Familienunternehmen in zweiter Generation mit Transporten, eigenem Fuhrpark, Lagerlogistik und Palettenmanagement im Westmünsterland. Kleinerer, aber voll ausgebauter Betrieb mit Dispo-, QM- und Projektmanagement-Funktionen; Hinweis: liegt vermutlich unterhalb der 50-Mitarbeiter-Schwelle.</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>https://hoeper-spedition.de/team/ | https://hoeper-spedition.de/ | https://hoeper-spedition.de/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Tanja Meininghaus</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Geschäftsführerin</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>tanja.meininghaus@sitra-spedition.de</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>+49 40 751006-0 (Zentrale)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>SITRA Spedition GmbH</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Inhabergeführte Hamburger Spedition mit nationalen Stückgut-/Ladungsverkehren, internationalem Geschäft und eigener Disposition; bewusst als persönlich erreichbare Alternative zu Konzernen positioniert.</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>https://sitra-spedition.de/team/ | https://sitra-spedition.de/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Sandra Aleksanderek</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Geschäftsführung</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>sandra.aleksanderek@sander-logistics.de</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>+49 40 73354-128</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Sander Logistics GmbH</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Hamburg (Altenwerder), weitere Standorte Itzehoe und Rostock</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Mittelständisches, familiengeführtes Logistikunternehmen mit Sammelgut, Komplettladungen, Seefracht sowie Lager-, Beschaffungs- und Kontraktlogistik an fünf Standorten.</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>https://sander-logistics.de/ihre-ansprechpartner/ | https://sander-logistics.de/kontakt/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Frank Blodt</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>frankblodt@spedition-blodt.de</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>+49 6131 25007-0</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Spedition Blodt GmbH</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Mainz, Rheinland-Pfalz</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Familiengeführte Spedition in Mainz mit Transport, Lagerlogistik und Projektmanagement; Geschäftsführung und Lagerlogistik liegen in der Familie Blodt.</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>https://spedition-blodt.de/unser-team/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Miriam Blodt</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Geschäftsführerin</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>miriamblodt@spedition-blodt.de</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>+49 6131 25007-0</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Spedition Blodt GmbH</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Mainz, Rheinland-Pfalz</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Zweite Geschäftsführerin des inhabergeführten Mainzer Speditions- und Lagerlogistikbetriebs.</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>https://spedition-blodt.de/unser-team/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Bernd Häger</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>bhaeger@spedition-haeger.de</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>02904 9740-0</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Spedition Häger GmbH &amp; Co. KG / Häger Transporte u. Logistik GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Bestwig (Sauerland, NRW)</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Familiengeführte Sauerland-Spedition mit Transport-, Lager- und Kontraktlogistik über zwei Schwestergesellschaften. Zwei-Firmen-Struktur und gewachsene Dispositions-/Lagerprozesse sprechen für manuelle Abläufe mit Digitalisierungs- und Systemintegrationsbedarf.</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.spedition-haeger.de/kontakt/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Nicole Körtge</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Leitung Auftragsmanagement/Logistik</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>nicolekoertge@spedition-wagner.net</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>+49 2642 9022922</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Spedition Wagner GmbH</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Remagen (Am Römerhof 60, 53424), Rheinland-Pfalz</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Familiengeführter Logistikdienstleister mit Kontraktlogistik für die Getränkeindustrie (u. a. Krombacher), Lagerlogistik, Displaybau und eigenem Fuhrpark. Geschäftsführung (Arlt/Gaßner/Kröhl) ohne öffentliche E-Mail – Bereichsleitung Logistik als Entscheidungsträger.</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>https://spedition-wagner.net/unternehmen/team/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Matthias Schork</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>m.schork@wuest.com</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>+49 9141 8684-140</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Spedition Wüst (Wüst GmbH &amp; Co. KG)</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Weißenburg i. Bay., weiteres Logistikzentrum Ansbach, Bayern</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Mittelständische bayerische Spedition mit Stückgut- und Ladungsverkehren sowie zwei eigenen Logistikzentren (Lagerung, Kommissionierung, Value Added Services).</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.wuest.com/kontakt/ | https://www.wuest.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Michael Müller</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Logistikleiter</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>m.mueller@wuest.com</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>+49 9141 8684-106</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Spedition Wüst (Wüst GmbH &amp; Co. KG)</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Weißenburg i. Bay., Bayern</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Verantwortlicher für die Logistikzentren Weißenburg und Ansbach – direkter Entscheider für Lager-/Kontraktlogistikprozesse.</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.wuest.com/kontakt/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Ralf Greinert</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>ralf.greinert@teamlogistic.de</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>+49 2602 1309-0 (Zentrale)</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>TEAM Logistic GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Montabaur (Westerwaldstr. 2a, 56410), Rheinland-Pfalz</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Familiengeführte Spedition im Westerwald (Familie Greinert) mit eigener Disposition, Werkstatt und Verwaltung; Transporte national/international.</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>https://teamlogistic.de/ansprechpartner/ | https://teamlogistic.de/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Uwe Diel</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>uwe.diel@teamlogistic.de</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>+49 2602 1309-0 (Zentrale)</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>TEAM Logistic GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Montabaur, Rheinland-Pfalz</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Zweiter Geschäftsführer der Team Logistic GmbH &amp; Co. KG, mittelständische Spedition mit eigenem Fuhrpark.</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>https://teamlogistic.de/ansprechpartner/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Theodor Schulz</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Geschäftsführer (Disposition &amp; Kundenbetreuung)</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>ts@schulz-spedition.de</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>+49 251 26333-211</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Theodor Schulz GmbH &amp; Co. KG (Schulz Spedition)</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Münster (NRW)</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Inhabergeführte Münsteraner Spedition mit Transport, Lagerung/Lagerverwaltung, Palettenmanagement und Abrechnung als eigene Abteilungen. Geschäftsführung sitzt selbst in der Disposition — kurze Entscheidungswege, viele manuell getriebene Dispo- und Abrechnungsprozesse als Digitalisierungsansatz.</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.schulz-spedition.de/ | https://www.schulz-spedition.de/#unternehmen</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
           <t>Christian Vetten</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Geschäftsführer (Ansprechpartner Transporte/Lagerlogistik)</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>christian.vetten@vetten-gruppe.de</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>02162 5302-379</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>Vetten Gruppe (Gebr. Vetten GmbH &amp; Co. KG)</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Logistik &amp; Supply Chain</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>Mönchengladbach (Niederrhein, NRW)</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>Familienbetrieb seit 1931 mit Transport, Lagerlogistik, Textil- und Kontraktlogistik auf &gt;100.000 qm Lagerfläche. Gewachsene Gruppenstruktur mit mehreren Standorten, Variantenvielfalt (Textilaufbereitung, Kontraktlogistik) und vorhandener Logistik-IT (ecovium/SPEDION im Einsatz) — viel Potenzial für Prozessdigitalisierung und Schnittstellen-/ERP-Themen.</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>https://vetten-gruppe.de/kontakt/ | https://vetten-gruppe.de/ | https://vetten-gruppe.de/impressum/ | https://vetten-gruppe.de/die-vetten-gruppe/</t>
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Andreas Koch</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>a.koch@eckhardt-logistik.de</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>+49 711 80000-0 (Zentrale)</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Walter Eckhardt GmbH Spedition + Logistik</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Korntal-Münchingen (Raum Stuttgart), Baden-Württemberg</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Inhabergeführte Spedition seit 1987 mit Stückgut, Gefahrgut- und Pflanzentransporten sowie eigenem Lager-/Kommissionierzentrum (seit 2019). Eigene Bereiche für Umschlag, Lagerlogistik und Disposition.</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>https://eckhardt-logistik.de/kontakt/ansprechpartner | https://eckhardt-logistik.de/</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Marc Eckhardt</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Gesellschafter (Inhaberfamilie)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>m.eckhardt@eckhardt-logistik.de</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>+49 711 80000-0 (Zentrale)</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Walter Eckhardt GmbH Spedition + Logistik</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Korntal-Münchingen (Raum Stuttgart), Baden-Württemberg</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Gesellschafter und Namensträger des familiengeführten Speditions- und Logistikunternehmens; zweiter Entscheidungsträger neben der Geschäftsführung.</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>https://eckhardt-logistik.de/kontakt/ansprechpartner | https://eckhardt-logistik.de/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I8"/>
+  <autoFilter ref="A1:I26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -893,10 +1739,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="C4" t="n">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5">
@@ -919,10 +1765,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="C6" t="n">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -936,7 +1782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -970,12 +1816,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Kraftverkehr Münsterland C. Weilke GmbH &amp; Co. KG</t>
+          <t>Hermann Ritter GmbH &amp; Co. KG (Ritter Spedition)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Greven</t>
+          <t>Feilitzsch-Zedtwitz, Bayern</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -985,19 +1831,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>nur info@weilke.de auf Website, keine Ansprechpartner-/Teamseite mit Personen-E-Mails gefunden</t>
+          <t>nur 40 Mitarbeiter (unter Zielgröße) und nur info@-Adresse</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Richter Spedition GmbH</t>
+          <t>Metzger Spedition GmbH</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Schwerte</t>
+          <t>Neu-Kupfer, Baden-Württemberg</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1007,19 +1853,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>nur info@richter-spedition.de, keine Personenseite; Geschäftsführung nicht mit E-Mail veröffentlicht</t>
+          <t>nur info@metzger-spedition.de, keine Personen auf der Website</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Gustav Mäuler GmbH &amp; Co. KG</t>
+          <t>Rüdinger Spedition GmbH</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Remscheid</t>
+          <t>Krautheim, Baden-Württemberg</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1029,19 +1875,19 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>nur info@ und verkauf@ (Funktionsadressen), keine namentlichen Ansprechpartner auf Homepage und Kontaktseite</t>
+          <t>Ansprechpartner mit Namen/Positionen, aber E-Mail-Adressen verschleiert; auch per curl keine Adresse im Quelltext</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Spedition Zobel</t>
+          <t>ZUFALL logistics group (Friedrich Zufall GmbH &amp; Co. KG)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Wetter (Ruhr)</t>
+          <t>Göttingen, Niedersachsen</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1051,19 +1897,19 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Ansprechpartner-Seite nennt nur Personalmanagement; keine E-Mail der Geschäftsführer Philip/Christian Zobel veröffentlicht</t>
+          <t>nur standortbezogene Sammeladressen (goettingen@, kassel@ …), keine persönliche E-Mail der Geschäftsführung</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LLS-Service GmbH</t>
+          <t>Heinrich Koch Internationale Spedition GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Gladbeck</t>
+          <t>Osnabrück, Niedersachsen</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1073,19 +1919,19 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>nur info@lls.services, keine namentlichen Entscheidungsträger auf der Website</t>
+          <t>auf der Kontaktseite nur info@koch-international.de, keine Ansprechpartner-Seite mit Personen-E-Mails</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Emmerich &amp; Rosenberger GmbH &amp; Co. KG (EMRO)</t>
+          <t>Döderlein Spedition GmbH</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Duisburg</t>
+          <t>Nördlingen, Bayern</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1095,19 +1941,19 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>nur info@emro.de, keine Ansprechpartner-Seite mit persönlichen E-Mails gefunden</t>
+          <t>nur info@doederlein.de, keine Ansprechpartner-/Teamseite</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NW Logistik</t>
+          <t>Elflein Spedition &amp; Transport GmbH</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Ahlen</t>
+          <t>Bamberg, Bayern</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1117,19 +1963,19 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Website nicht erreichbar (DNS-Fehler), keine Daten verifizierbar</t>
+          <t>Geschäftsführer mit Durchwahl gelistet, aber E-Mail-Links leer ('#') – keine wörtliche Adresse auf der Seite</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Emons Spedition GmbH</t>
+          <t>Spedicam GmbH</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Köln</t>
+          <t>Neufahrn (Raum München), Bayern</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1139,27 +1985,555 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Konzernähnliche Größe (&gt;3.000 Mitarbeiter, 100 Standorte) — außerhalb Mittelstands-Zielprofil</t>
+          <t>nur Funktionsadressen (Gf@, Sl@, Vl@ …), keine personenbezogenen E-Mails</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Wiedmann &amp; Winz GmbH</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Geislingen an der Steige, Baden-Württemberg</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>nur Funktionsadressen (mail@, offer@, anfrage@), keine Ansprechpartner-Seite</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BKV Logistik GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Rheinstetten, Baden-Württemberg</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>nur Funktionsadressen (kontakt@, transportlogistik@, kontraktlogistik@)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BECK Spedition + Logistik GmbH</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Filderstadt, Baden-Württemberg</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>nur info@becksped.de, keine Personen auf der Kontaktseite</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Abt Spedition &amp; Service</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Schwäbisch Gmünd, Baden-Württemberg</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Ansprechpartner Jochen Abt genannt, aber nur info@abt-spedition.de</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Honold Contract Logistics GmbH</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Neu-Ulm, Bayern</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Geschäftsführer namentlich genannt, aber nur Sammeladresse kontraktlogistik@honold.net</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>LTG Logistik und Transport GmbH</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>keine E-Mail-Adressen auf der Kontaktseite</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>RM Logistik GmbH</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Grasberg / Bremen</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Geschäftsführung (Familie Meyer) mit Telefon, aber keine E-Mail-Adressen auf der Seite</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Spedition Bode GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Bad Oldesloe/Bargteheide, Schleswig-Holstein</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>persönliche GF-Adresse vorhanden, aber Standort außerhalb der definierten Zielregionen</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Finsterwalder Transport &amp; Logistik GmbH</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Türkheim, Bayern</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>nur standortbezogene Sammeladressen (sales.tu@ …)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Noerpel-Gruppe</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Ulm / Hamburg / Hannover</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>über 1.000 Mitarbeiter, außerhalb der Zielgröße; nur info@noerpel.de</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Rudolph Logistik Gruppe</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Gudensberg, Hessen</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>ca. 4.500 Mitarbeiter an 42 Standorten – Konzerngröße, außerhalb Zielprofil</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>LOXXESS AG</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Tegernsee, Bayern</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Kontraktlogistiker deutlich über 1.000 Mitarbeitern – außerhalb Zielgröße</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Spedition König</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Esslingen, Baden-Württemberg</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>nur info@koenig-sped.de</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Spedition Kübler GmbH</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Michelfeld/Schwäbisch Hall, Baden-Württemberg</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>nur info@kuebler-spedition.de, keine personenbezogenen E-Mails</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>E3 Spedition (E3 Gruppe)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Homberg (Hessen) u. a.</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Ansprechpartner nur über JavaScript-Filter, keine E-Mails im Seitenquelltext</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Carl Köster &amp; Louis Hapke – Kontaktseite</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Sehnde-Höver, Niedersachsen</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Hinweis: /kontakt/ enthält nur info@; verwertbare Daten ausschließlich auf /ansprechpartner/ (siehe Lead)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Kraftverkehr Münsterland C. Weilke GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Greven</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>nur info@weilke.de auf Website, keine Ansprechpartner-/Teamseite mit Personen-E-Mails gefunden</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Richter Spedition GmbH</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Schwerte</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>nur info@richter-spedition.de, keine Personenseite; Geschäftsführung nicht mit E-Mail veröffentlicht</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Gustav Mäuler GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Remscheid</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>nur info@ und verkauf@ (Funktionsadressen), keine namentlichen Ansprechpartner auf Homepage und Kontaktseite</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Spedition Zobel</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Wetter (Ruhr)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Ansprechpartner-Seite nennt nur Personalmanagement; keine E-Mail der Geschäftsführer Philip/Christian Zobel veröffentlicht</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>LLS-Service GmbH</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Gladbeck</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>nur info@lls.services, keine namentlichen Entscheidungsträger auf der Website</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Emmerich &amp; Rosenberger GmbH &amp; Co. KG (EMRO)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Duisburg</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>nur info@emro.de, keine Ansprechpartner-Seite mit persönlichen E-Mails gefunden</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>NW Logistik</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Ahlen</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Website nicht erreichbar (DNS-Fehler), keine Daten verifizierbar</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Emons Spedition GmbH</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Köln</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Konzernähnliche Größe (&gt;3.000 Mitarbeiter, 100 Standorte) — außerhalb Mittelstands-Zielprofil</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>TEAM Logistic (Greinert/Diel)</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>Raum Montabaur (RLP)</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Logistik &amp; Supply Chain</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Logistik &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
         <is>
           <t>persönliche GF-E-Mails vorhanden, aber außerhalb Zielregion und Größe nicht verifiziert — nachqualifizierbar</t>
         </is>

</xml_diff>